<commit_message>
Shrink Sheet Lab access spreadsheet for Google Drive upload
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NfiPPgsq2NdhWywDYUoWaR
</commit_message>
<xml_diff>
--- a/The_Sheet_Lab_Access.xlsx
+++ b/The_Sheet_Lab_Access.xlsx
@@ -51,17 +51,12 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -81,19 +76,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -491,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="B13:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -503,221 +497,43 @@
     <col width="4" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="1" t="n"/>
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-      <c r="G3" s="1" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="1" t="n"/>
-      <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n"/>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="1" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="1" t="n"/>
-      <c r="B7" s="1" t="n"/>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="1" t="n"/>
-      <c r="D10" s="1" t="n"/>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="n"/>
-      <c r="G10" s="1" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="1" t="n"/>
-      <c r="D11" s="1" t="n"/>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="1" t="n"/>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
-    </row>
+    <row r="2" ht="18" customHeight="1"/>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Click here to access your Google Sheet</t>
         </is>
       </c>
-      <c r="G13" s="1" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="1" t="n"/>
-      <c r="C14" s="1" t="n"/>
-      <c r="D14" s="1" t="n"/>
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
     </row>
     <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="1" t="n"/>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>⬇</t>
         </is>
       </c>
-      <c r="G15" s="1" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="1" t="n"/>
     </row>
     <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="1" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>👉 OPEN YOUR GOOGLE SHEET 👈</t>
         </is>
       </c>
-      <c r="G17" s="1" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n"/>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
-      <c r="G18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n"/>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Thank you for your purchase — The Sheet Lab</t>
         </is>
       </c>
-      <c r="G19" s="1" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n"/>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
-      <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="n"/>
-      <c r="G20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n"/>
-      <c r="B21" s="1" t="n"/>
-      <c r="C21" s="1" t="n"/>
-      <c r="D21" s="1" t="n"/>
-      <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="n"/>
-      <c r="G21" s="1" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n"/>
-      <c r="B22" s="1" t="n"/>
-      <c r="C22" s="1" t="n"/>
-      <c r="D22" s="1" t="n"/>
-      <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n"/>
-      <c r="B23" s="1" t="n"/>
-      <c r="C23" s="1" t="n"/>
-      <c r="D23" s="1" t="n"/>
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-      <c r="G23" s="1" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
-      <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Redesign Sheet Lab access page with new logo and centered layout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NfiPPgsq2NdhWywDYUoWaR
</commit_message>
<xml_diff>
--- a/The_Sheet_Lab_Access.xlsx
+++ b/The_Sheet_Lab_Access.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,27 +28,37 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3A5F"/>
-      <sz val="20"/>
+      <color rgb="002EC88C"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002E9E5B"/>
-      <sz val="48"/>
+      <color rgb="000F1821"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="006B7785"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002EC88C"/>
+      <sz val="40"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="007F8C8D"/>
-      <sz val="10"/>
+      <color rgb="009AA4AF"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,7 +70,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E9E5B"/>
+        <fgColor rgb="001C9B6C"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,19 +86,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -170,12 +186,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>2</col>
-      <colOff>619125</colOff>
+      <col>1</col>
+      <colOff>1714500</colOff>
       <row>1</row>
-      <rowOff>0</rowOff>
+      <rowOff>76200</rowOff>
     </from>
-    <ext cx="1714500" cy="1743075"/>
+    <ext cx="2286000" cy="2286000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -485,65 +501,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B13:F19"/>
+  <dimension ref="B3:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="18" customHeight="1"/>
-    <row r="3" ht="18" customHeight="1"/>
-    <row r="4" ht="18" customHeight="1"/>
-    <row r="5" ht="18" customHeight="1"/>
-    <row r="6" ht="18" customHeight="1"/>
-    <row r="7" ht="18" customHeight="1"/>
-    <row r="8" ht="18" customHeight="1"/>
-    <row r="9" ht="18" customHeight="1"/>
-    <row r="10" ht="18" customHeight="1"/>
-    <row r="11" ht="18" customHeight="1"/>
-    <row r="13" ht="40" customHeight="1">
-      <c r="B13" s="1" t="inlineStr">
+    <row r="1" ht="20" customHeight="1"/>
+    <row r="2" ht="192" customHeight="1"/>
+    <row r="3" ht="26" customHeight="1">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Thank you for your purchase!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Click here to access your Google Sheet</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="70" customHeight="1">
-      <c r="B15" s="2" t="inlineStr">
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Use the button below to open your copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>⬇</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="7" ht="46" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>👉 OPEN YOUR GOOGLE SHEET 👈</t>
+          <t>OPEN YOUR GOOGLE SHEET</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Thank you for your purchase — The Sheet Lab</t>
+          <t>The Sheet Lab  •  Financial Tools</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B19:F19"/>
-  </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>

</xml_diff>